<commit_message>
Update forecast data and fix deploy script
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B925"/>
+  <dimension ref="A1:B926"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7763,6 +7763,14 @@
         <v>4.86965</v>
       </c>
     </row>
+    <row r="926" spans="1:2">
+      <c r="A926" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B926">
+        <v>4.84211</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-05-30_18-04-58
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B926"/>
+  <dimension ref="A1:B927"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7771,6 +7771,14 @@
         <v>4.84211</v>
       </c>
     </row>
+    <row r="927" spans="1:2">
+      <c r="A927" s="2">
+        <v>46171</v>
+      </c>
+      <c r="B927">
+        <v>4.85786</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-06-06_09-10-56
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B927"/>
+  <dimension ref="A1:B928"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7779,6 +7779,14 @@
         <v>4.85786</v>
       </c>
     </row>
+    <row r="928" spans="1:2">
+      <c r="A928" s="2">
+        <v>46178</v>
+      </c>
+      <c r="B928">
+        <v>4.78426</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-06-13_11-28-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B928"/>
+  <dimension ref="A1:B929"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7787,6 +7787,14 @@
         <v>4.78426</v>
       </c>
     </row>
+    <row r="929" spans="1:2">
+      <c r="A929" s="2">
+        <v>46185</v>
+      </c>
+      <c r="B929">
+        <v>4.76339</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-06-28_10-57-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B930"/>
+  <dimension ref="A1:B931"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7829,6 +7829,14 @@
         <v>4.75535</v>
       </c>
     </row>
+    <row r="931" spans="1:2">
+      <c r="A931" s="3">
+        <v>46199</v>
+      </c>
+      <c r="B931">
+        <v>4.69327</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-07-12_00-02-05
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B931"/>
+  <dimension ref="A1:B933"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7837,6 +7837,22 @@
         <v>4.69327</v>
       </c>
     </row>
+    <row r="932" spans="1:2">
+      <c r="A932" s="3">
+        <v>46206</v>
+      </c>
+      <c r="B932">
+        <v>4.70817</v>
+      </c>
+    </row>
+    <row r="933" spans="1:2">
+      <c r="A933" s="3">
+        <v>46213</v>
+      </c>
+      <c r="B933">
+        <v>4.713</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-07-14_20-36-16
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B933"/>
+  <dimension ref="A1:B934"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7853,6 +7853,14 @@
         <v>4.713</v>
       </c>
     </row>
+    <row r="934" spans="1:2">
+      <c r="A934" s="3">
+        <v>46220</v>
+      </c>
+      <c r="B934">
+        <v>4.69175</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-07-21_14-43-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B934"/>
+  <dimension ref="A1:B935"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7861,6 +7861,14 @@
         <v>4.73111</v>
       </c>
     </row>
+    <row r="935" spans="1:2">
+      <c r="A935" s="3">
+        <v>46227</v>
+      </c>
+      <c r="B935">
+        <v>4.73382</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-07-28_20-35-15
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B935"/>
+  <dimension ref="A1:B936"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7869,6 +7869,14 @@
         <v>4.7259</v>
       </c>
     </row>
+    <row r="936" spans="1:2">
+      <c r="A936" s="3">
+        <v>46234</v>
+      </c>
+      <c r="B936">
+        <v>4.7282</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-08-04_20-32-59
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B936"/>
+  <dimension ref="A1:B937"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7877,6 +7877,14 @@
         <v>4.74093</v>
       </c>
     </row>
+    <row r="937" spans="1:2">
+      <c r="A937" s="3">
+        <v>46241</v>
+      </c>
+      <c r="B937">
+        <v>4.72932</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-08-11_20-42-32
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B937"/>
+  <dimension ref="A1:B938"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7885,6 +7885,14 @@
         <v>4.76528</v>
       </c>
     </row>
+    <row r="938" spans="1:2">
+      <c r="A938" s="3">
+        <v>46248</v>
+      </c>
+      <c r="B938">
+        <v>4.75742</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-08-18_20-33-31
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B938"/>
+  <dimension ref="A1:B939"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7893,6 +7893,14 @@
         <v>4.77564</v>
       </c>
     </row>
+    <row r="939" spans="1:2">
+      <c r="A939" s="3">
+        <v>46255</v>
+      </c>
+      <c r="B939">
+        <v>4.78877</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-08-25_20-33-34
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B939"/>
+  <dimension ref="A1:B940"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7901,6 +7901,14 @@
         <v>4.81707</v>
       </c>
     </row>
+    <row r="940" spans="1:2">
+      <c r="A940" s="3">
+        <v>46262</v>
+      </c>
+      <c r="B940">
+        <v>4.80441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-09-01_20-36-02
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B940"/>
+  <dimension ref="A1:B941"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7909,6 +7909,14 @@
         <v>4.81815</v>
       </c>
     </row>
+    <row r="941" spans="1:2">
+      <c r="A941" s="3">
+        <v>46269</v>
+      </c>
+      <c r="B941">
+        <v>4.81398</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>